<commit_message>
updated example and switched to standard style to keep things as simple as possible.
</commit_message>
<xml_diff>
--- a/examples/responses/1_daisy_jr-woodchucks.xlsx
+++ b/examples/responses/1_daisy_jr-woodchucks.xlsx
@@ -762,7 +762,7 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>META.Q1</t>
+          <t>USG.Q1</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -782,7 +782,7 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>META.Q2</t>
+          <t>USG.Q2</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>META.Q3</t>
+          <t>USG.Q3</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -819,14 +819,14 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Options: YAML-configured Excel (umfrage), Web forms (e.g., LimeSurvey, SurveyMonkey), Paper forms, LaTeX-compiled PDF, Other</t>
+          <t>Choose your preferred distribution format from the dropdown</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>META.Q4</t>
+          <t>USG.Q4</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -876,7 +876,7 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>META.Q5</t>
+          <t>REQ.Q1</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -896,7 +896,7 @@
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>META.Q6</t>
+          <t>REQ.Q2</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -916,7 +916,7 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>META.Q7</t>
+          <t>REQ.Q3</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -938,7 +938,7 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>META.Q8</t>
+          <t>REQ.Q4</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -953,14 +953,14 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Options: Automated result aggregation, Data validation / input dropdowns, Protected / tamper-evident forms, Version control compatibility, Offline use without internet access</t>
+          <t>Select the single most critical feature from the dropdown</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>META.Q9</t>
+          <t>REQ.Q5</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>90e431d2cf00dd3bdc3db465c656595a22edbad47eeddbb4330f0576b1f74ba0</t>
+          <t>936da7177b2b9ee7a3df989da45111cb279720c784ea31e6188567aa11660488</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-25T10:19:56.229788+00:00</t>
+          <t>2026-08-26T14:20:27.626404+00:00</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>["META.Q1", "META.Q2", "META.Q3", "META.Q4", "META.Q5", "META.Q6", "META.Q7", "META.Q8", "META.Q9"]</t>
+          <t>["USG.Q1", "USG.Q2", "USG.Q3", "USG.Q4", "REQ.Q1", "REQ.Q2", "REQ.Q3", "REQ.Q4", "REQ.Q5"]</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"title":"Survey Tools in Research — A Meta-Survey","version":"1.0","language":"en","choice_lists":{"questionnaire_format":["YAML-configured Excel (umfrage)","Web forms (e.g., LimeSurvey, SurveyMonkey)","Paper forms","LaTeX-compiled PDF","Other"],"critical_feature":["Automated result aggregation","Data validation / input dropdowns","Protected / tamper-evident forms","Version control compatibility","Offline use without internet access"]},"organizer":{"name":"Prof. Dr. Ludwig von Drake","institution":"Duckburg Academy of Sciences","email":"l.von-drake@duckburg.edu","phone":null},"respondent_fields":[{"label":"Name","required":true},{"label":"Institution","required":true},{"label":"Email","required":false}],"sections":[{"title":"Usage Patterns","questions":[{"id":"META.Q1","text":"How frequently do you design or distribute questionnaires in your work?","answer":{"type":"scale","min_value":1,"max_value":5,"description":"1 = rarely or never, 5 = regularly, multiple times per year","choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"META.Q2","text":"Does your institution currently use Excel-based survey forms (rather than web-based)?","answer":{"type":"yes_no","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"META.Q3","text":"Which questionnaire distribution format do you prefer?","answer":{"type":"choices","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":"questionnaire_format","show_choices_in_comment":true},"comment":null,"required":true},{"id":"META.Q4","text":"If you have a preferred survey tool, please name it.","answer":{"type":"freetext","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":false}]},{"title":"Tool Requirements","questions":[{"id":"META.Q5","text":"How important is it for a questionnaire tool to be freely available and open-source?","answer":{"type":"scale","min_value":1,"max_value":5,"description":"1 = irrelevant, 5 = essential","choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"META.Q6","text":"How important is consistent layout reproduction across all recipient workstations?","answer":{"type":"scale","min_value":1,"max_value":5,"description":"1 = irrelevant, 5 = essential","choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"META.Q7","text":"Would you accept defining questionnaires in a structured text format such as YAML?","answer":{"type":"yes_no","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"META.Q8","text":"Which tool feature do you consider most critical?","answer":{"type":"choices","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":"critical_feature","show_choices_in_comment":true},"comment":null,"required":true},{"id":"META.Q9","text":"Any additional requirements, comments, or suggestions?","answer":{"type":"freetext","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":false}]}]}</t>
+          <t>{"title":"Survey Tools in Research — A Meta-Survey","version":"1.0","language":"en","choice_lists":{"questionnaire_format":["YAML-configured Excel (umfrage)","Web forms (e.g., LimeSurvey, SurveyMonkey)","Paper forms","LaTeX-compiled PDF","Other"],"critical_feature":["Automated result aggregation","Data validation / input dropdowns","Protected / tamper-evident forms","Version control compatibility","Offline use without internet access"]},"organizer":{"name":"Prof. Dr. Ludwig von Drake","institution":"Duckburg Academy of Sciences","email":"l.von-drake@duckburg.edu","phone":null},"respondent_fields":[{"label":"Name","required":true},{"label":"Institution","required":true},{"label":"Email","required":false}],"sections":[{"title":"Usage Patterns","questions":[{"id":"USG.Q1","text":"How frequently do you design or distribute questionnaires in your work?","answer":{"type":"scale","min_value":1,"max_value":5,"description":"1 = rarely or never, 5 = regularly, multiple times per year","choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"USG.Q2","text":"Does your institution currently use Excel-based survey forms (rather than web-based)?","answer":{"type":"yes_no","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"USG.Q3","text":"Which questionnaire distribution format do you prefer?","answer":{"type":"choices","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":"questionnaire_format","show_choices_in_comment":true},"comment":"Choose your preferred distribution format from the dropdown","required":true},{"id":"USG.Q4","text":"If you have a preferred survey tool, please name it.","answer":{"type":"freetext","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":false}]},{"title":"Tool Requirements","questions":[{"id":"REQ.Q1","text":"How important is it for a questionnaire tool to be freely available and open-source?","answer":{"type":"scale","min_value":1,"max_value":5,"description":"1 = irrelevant, 5 = essential","choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"REQ.Q2","text":"How important is consistent layout reproduction across all recipient workstations?","answer":{"type":"scale","min_value":1,"max_value":5,"description":"1 = irrelevant, 5 = essential","choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"REQ.Q3","text":"Would you accept defining questionnaires in a structured text format such as YAML?","answer":{"type":"yes_no","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":true},{"id":"REQ.Q4","text":"Which tool feature do you consider most critical?","answer":{"type":"choices","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":"critical_feature","show_choices_in_comment":true},"comment":"Select the single most critical feature from the dropdown","required":true},{"id":"REQ.Q5","text":"Any additional requirements, comments, or suggestions?","answer":{"type":"freetext","min_value":null,"max_value":null,"description":null,"choices":null,"choices_ref":null,"show_choices_in_comment":true},"comment":null,"required":false}]}]}</t>
         </is>
       </c>
     </row>

</xml_diff>